<commit_message>
feat(manuscripts): streamline candidate model suite, plain-English qualitative tone, and table synchronization
</commit_message>
<xml_diff>
--- a/results/04_model_execution_2025_holdout/04_model_execution_2025_holdout.xlsx
+++ b/results/04_model_execution_2025_holdout/04_model_execution_2025_holdout.xlsx
@@ -670,7 +670,7 @@
     <row r="2" ht="19" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>Baseline Control</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Diurnal Volatility Naive (y_{t-24})</t>
+          <t>Daily Persistence Benchmark (y_{t-24})</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -708,17 +708,17 @@
     <row r="3" ht="19" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
-          <t>M1*</t>
+          <t>Model 1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Deterministic Baseline</t>
+          <t>Deterministic Schedule</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Deterministic Schedule Bank Volatility Baseline</t>
+          <t>Deterministic Flight Schedule Model (convolved show-up curve)</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -746,17 +746,17 @@
     <row r="4" ht="19" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>Model 2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Probabilistic / ML</t>
+          <t>Machine Learning</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Supervised Volatility GBR (Combined Values + Vol)</t>
+          <t>Supervised Machine Learning Model (Decision Trees &amp; OTP)</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -784,7 +784,7 @@
     <row r="5" ht="19" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>Model 3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sequential SARIMA-Tree Volatility Hybrid</t>
+          <t>Dynamic Two-Stage Hybrid Model (Schedule + Real-time feedback)</t>
         </is>
       </c>
       <c r="D5" t="n">

</xml_diff>